<commit_message>
BIS-2185: Update reference data
</commit_message>
<xml_diff>
--- a/app-ro-crate-openbis/resources/metadata.xlsx
+++ b/app-ro-crate-openbis/resources/metadata.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="219">
   <si>
     <t>VOCABULARY_TYPE</t>
   </si>
@@ -96,17 +96,14 @@
   </si>
   <si>
     <t>schema.org
-http://datacite.org
 schema.org</t>
   </si>
   <si>
     <t>https://schema.org/Person
-http://datacite.org/schema/kernel-4#Creator
 https://schema.org/Author</t>
   </si>
   <si>
     <t>https://schema.org/version/28.1
-https://schema.datacite.org/meta/kernel-4.6/
 https://schema.org/version/28.1</t>
   </si>
   <si>
@@ -159,250 +156,227 @@
   </si>
   <si>
     <t>VARCHAR</t>
+  </si>
+  <si>
+    <t>schema.org</t>
+  </si>
+  <si>
+    <t>https://schema.org/identifier</t>
+  </si>
+  <si>
+    <t>https://schema.org/version/28.1</t>
+  </si>
+  <si>
+    <t>PUBLICATION_CREATOR.IDENTIFIER_SCHEME</t>
+  </si>
+  <si>
+    <t>Identifier Scheme</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>https://schema.org/name</t>
+  </si>
+  <si>
+    <t>PUBLICATION_CREATOR.GIVEN_NAME</t>
+  </si>
+  <si>
+    <t>Given Name</t>
+  </si>
+  <si>
+    <t>https://schema.org/givenName</t>
+  </si>
+  <si>
+    <t>PUBLICATION_CREATOR.FAMILY_NAME</t>
+  </si>
+  <si>
+    <t>Family Name</t>
+  </si>
+  <si>
+    <t>https://schema.org/familyName</t>
+  </si>
+  <si>
+    <t>PUBLICATION_CREATOR.AFFILITION_IDENTIFIER</t>
+  </si>
+  <si>
+    <t>Affilition</t>
+  </si>
+  <si>
+    <t>Affiliation Identifier</t>
+  </si>
+  <si>
+    <t>PUBLICATION_CREATOR.AFFILITION_IDENTIFIER_SCHEME</t>
+  </si>
+  <si>
+    <t>Affiliation Identifier Scheme</t>
+  </si>
+  <si>
+    <t>PUBLICATION_CREATOR.AFFILITION_IDENTIFIER_SCHEME_URI</t>
+  </si>
+  <si>
+    <t>Affiliation Identifier Scheme URI</t>
+  </si>
+  <si>
+    <t>PUBLICATION_PUBLISHER</t>
+  </si>
+  <si>
+    <t>PUBPUB</t>
+  </si>
+  <si>
+    <t>https://schema.org/</t>
+  </si>
+  <si>
+    <t>https://schema.org/Organization</t>
+  </si>
+  <si>
+    <t>PUBLICATION_PUBLISHER.IDENTIFIER</t>
+  </si>
+  <si>
+    <t>Publisher Identifier</t>
+  </si>
+  <si>
+    <t>PUBLICATION_PUBLISHER.IDENTIFIER_SCHEME</t>
+  </si>
+  <si>
+    <t>PUBLICATION_PUBLISHER.IDENTIFIER_SCHEME_URI</t>
+  </si>
+  <si>
+    <t>Identifier Scheme URI</t>
+  </si>
+  <si>
+    <t>PUBLICATION</t>
+  </si>
+  <si>
+    <t>PUB</t>
+  </si>
+  <si>
+    <t>https://schema.org/CreativeWork</t>
+  </si>
+  <si>
+    <t>ttps://schema.org/version/28.1</t>
+  </si>
+  <si>
+    <t>PUBLICATION.ORGANIZATION</t>
+  </si>
+  <si>
+    <t>Organization</t>
+  </si>
+  <si>
+    <t>http://schema.org/Organization</t>
+  </si>
+  <si>
+    <t>PUBLICATION.TYPE</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>PUBLICATION.IDENTIFIER</t>
+  </si>
+  <si>
+    <t>Publication Identifier</t>
+  </si>
+  <si>
+    <t>PUBLICATION.URL</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>HYPERLINK</t>
+  </si>
+  <si>
+    <t>https://schema.org/url</t>
+  </si>
+  <si>
+    <t>PUBLICATION.DESCRIPTION</t>
+  </si>
+  <si>
+    <t>https://schema.org/description</t>
+  </si>
+  <si>
+    <t>PUBLICATION.OPENBIS_RELATED_IDENTIFIERS</t>
+  </si>
+  <si>
+    <t>openBIS Related Identifiers</t>
+  </si>
+  <si>
+    <t>http://datacite.org</t>
+  </si>
+  <si>
+    <t>http://datacite.org/schema/kernel-4#relatedIdentifiers</t>
+  </si>
+  <si>
+    <t>https://schema.datacite.org/meta/kernel-4.6/</t>
+  </si>
+  <si>
+    <t>XMLCOMMENTS</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>XML</t>
+  </si>
+  <si>
+    <t>Comments log</t>
+  </si>
+  <si>
+    <t>PUBLICATION.STATUS</t>
+  </si>
+  <si>
+    <t>Publication Status</t>
+  </si>
+  <si>
+    <t>schema.org
+http://datacite.org</t>
+  </si>
+  <si>
+    <t>https://schema.org/creativeWorkStatus
+http://datacite.org/schema/kernel-4#stateSelection</t>
+  </si>
+  <si>
+    <t>https://schema.org/version/28.1
+https://schema.datacite.org/meta/kernel-4.6/</t>
+  </si>
+  <si>
+    <t>PUBLICATION.CONTRIBUTOR</t>
+  </si>
+  <si>
+    <t>Contributors</t>
+  </si>
+  <si>
+    <t>http://datacite.org/schema/kernel-4#doi</t>
+  </si>
+  <si>
+    <t>PUBLICATION.PUBLICATION_YEAR</t>
+  </si>
+  <si>
+    <t>Publication Year</t>
+  </si>
+  <si>
+    <t>TIMESTAMP</t>
   </si>
   <si>
     <t>http://datacite.org
 schema.org</t>
   </si>
   <si>
-    <t>http://datacite.org/schema/kernel-4#nameIdentifier
-https://schema.org/identifier</t>
+    <t>http://datacite.org/schema/kernel-4#publicationYear
+https://schema.org/datePublished</t>
   </si>
   <si>
     <t>https://schema.datacite.org/meta/kernel-4.6/
 https://schema.org/version/28.1</t>
   </si>
   <si>
-    <t>PUBLICATION_CREATOR.IDENTIFIER_SCHEME</t>
-  </si>
-  <si>
-    <t>Identifier Scheme</t>
-  </si>
-  <si>
-    <t>Identifier</t>
-  </si>
-  <si>
-    <t>NAME</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>schema.org</t>
-  </si>
-  <si>
-    <t>https://schema.org/name</t>
-  </si>
-  <si>
-    <t>https://schema.org/version/28.1</t>
-  </si>
-  <si>
-    <t>PUBLICATION_CREATOR.GIVEN_NAME</t>
-  </si>
-  <si>
-    <t>Given Name</t>
-  </si>
-  <si>
-    <t>schema.org
-http://datacite.org</t>
-  </si>
-  <si>
-    <t>https://schema.org/givenName
-http://datacite.org/schema/kernel-4#givenName</t>
-  </si>
-  <si>
-    <t>https://schema.org/version/28.1
-https://schema.datacite.org/meta/kernel-4.6/</t>
-  </si>
-  <si>
-    <t>PUBLICATION_CREATOR.FAMILY_NAME</t>
-  </si>
-  <si>
-    <t>Family Name</t>
-  </si>
-  <si>
-    <t>https://schema.org/familyName
-http://datacite.org/schema/kernel-4#familyName</t>
-  </si>
-  <si>
-    <t>PUBLICATION_CREATOR.AFFILITION_IDENTIFIER</t>
-  </si>
-  <si>
-    <t>Affilition</t>
-  </si>
-  <si>
-    <t>Affiliation Identifier</t>
-  </si>
-  <si>
-    <t>PUBLICATION_CREATOR.AFFILITION_IDENTIFIER_SCHEME</t>
-  </si>
-  <si>
-    <t>Affiliation Identifier Scheme</t>
-  </si>
-  <si>
-    <t>PUBLICATION_CREATOR.AFFILITION_IDENTIFIER_SCHEME_URI</t>
-  </si>
-  <si>
-    <t>Affiliation Identifier Scheme URI</t>
-  </si>
-  <si>
-    <t>PUBLICATION_PUBLISHER</t>
-  </si>
-  <si>
-    <t>PUBPUB</t>
-  </si>
-  <si>
-    <t>https://schema.org/</t>
-  </si>
-  <si>
-    <t>https://schema.org/Organization</t>
-  </si>
-  <si>
-    <t>PUBLICATION_PUBLISHER.IDENTIFIER</t>
-  </si>
-  <si>
-    <t>Publisher Identifier</t>
-  </si>
-  <si>
-    <t>https://schema.org/identifier
-http://datacite.org/schema/kernel-4#publisherIdentifier</t>
-  </si>
-  <si>
-    <t>PUBLICATION_PUBLISHER.IDENTIFIER_SCHEME</t>
-  </si>
-  <si>
-    <t>http://datacite.org</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#publisherIdentifierScheme</t>
-  </si>
-  <si>
-    <t>https://schema.datacite.org/meta/kernel-4.6/</t>
-  </si>
-  <si>
-    <t>PUBLICATION_PUBLISHER.IDENTIFIER_SCHEME_URI</t>
-  </si>
-  <si>
-    <t>Identifier Scheme URI</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#schemeURI</t>
-  </si>
-  <si>
-    <t>PUBLICATION</t>
-  </si>
-  <si>
-    <t>PUB</t>
-  </si>
-  <si>
-    <t>https://schema.org/CreativeWork</t>
-  </si>
-  <si>
-    <t>ttps://schema.org/version/28.1</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#title
-https://schema.org/name</t>
-  </si>
-  <si>
-    <t>PUBLICATION.ORGANIZATION</t>
-  </si>
-  <si>
-    <t>Organization</t>
-  </si>
-  <si>
-    <t>http://schema.org/Organization</t>
-  </si>
-  <si>
-    <t>PUBLICATION.TYPE</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>PUBLICATION.IDENTIFIER</t>
-  </si>
-  <si>
-    <t>Publication Identifier</t>
-  </si>
-  <si>
-    <t>https://schema.org/identifier
-http://datacite.org/schema/kernel-4#doi</t>
-  </si>
-  <si>
-    <t>PUBLICATION.URL</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>HYPERLINK</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#url
-https://schema.org/url</t>
-  </si>
-  <si>
-    <t>PUBLICATION.DESCRIPTION</t>
-  </si>
-  <si>
-    <t>https://schema.org/description
-http://datacite.org/schema/kernel-4#descriptions</t>
-  </si>
-  <si>
-    <t>PUBLICATION.OPENBIS_RELATED_IDENTIFIERS</t>
-  </si>
-  <si>
-    <t>openBIS Related Identifiers</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#relatedIdentifiers</t>
-  </si>
-  <si>
-    <t>XMLCOMMENTS</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>XML</t>
-  </si>
-  <si>
-    <t>Comments log</t>
-  </si>
-  <si>
-    <t>PUBLICATION.STATUS</t>
-  </si>
-  <si>
-    <t>Publication Status</t>
-  </si>
-  <si>
-    <t>https://schema.org/creativeWorkStatus
-http://datacite.org/schema/kernel-4#stateSelection</t>
-  </si>
-  <si>
-    <t>PUBLICATION.CONTRIBUTOR</t>
-  </si>
-  <si>
-    <t>Contributors</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#doi</t>
-  </si>
-  <si>
-    <t>PUBLICATION.PUBLICATION_YEAR</t>
-  </si>
-  <si>
-    <t>Publication Year</t>
-  </si>
-  <si>
-    <t>TIMESTAMP</t>
-  </si>
-  <si>
-    <t>http://datacite.org/schema/kernel-4#publicationYear
-https://schema.org/datePublished</t>
-  </si>
-  <si>
     <t>PUBLICATION.CREATOR</t>
   </si>
   <si>
@@ -523,21 +497,54 @@
     <t>Children</t>
   </si>
   <si>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUB29</t>
+  </si>
+  <si>
+    <t>PUB29</t>
+  </si>
+  <si>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_COLLECTION</t>
+  </si>
+  <si>
+    <t>Genetic mechanisms of critical illness in COVID-19</t>
+  </si>
+  <si>
+    <t>DataPaper</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41586-020-03065-y</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41586-020-03065-y#citeas</t>
+  </si>
+  <si>
+    <t>Genetic mechanisms of critical illness in COVID-19 for testing purposes</t>
+  </si>
+  <si>
+    <t>Registered</t>
+  </si>
+  <si>
+    <t>2020-12-11 14:48:55 +0000</t>
+  </si>
+  <si>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBCREA23</t>
+  </si>
+  <si>
+    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBPUB26</t>
+  </si>
+  <si>
+    <t>Host-mediated lung inflammation is present1, and drives mortality2, in the critical illness caused by coronavirus disease 2019 (COVID-19). Host genetic variants associated with critical illness may identify mechanistic targets for therapeutic development3. Here we report the results of the GenOMICC (Genetics Of Mortality In Critical Care) genome-wide association study in 2,244 critically ill patients with COVID-19 from 208 UK intensive care units. We have identified and replicated the following new genome-wide significant associations: on chromosome 12q24.13 (rs10735079, P = 1.65 × 10−8) in a gene cluster that encodes antiviral restriction enzyme activators (OAS1, OAS2 and OAS3); on chromosome 19p13.2 (rs74956615, P = 2.3 × 10−8) near the gene that encodes tyrosine kinase 2 (TYK2); on chromosome 19p13.3 (rs2109069, P = 3.98 ×  10−12) within the gene that encodes dipeptidyl peptidase 9 (DPP9); and on chromosome 21q22.1 (rs2236757, P = 4.99 × 10−8) in the interferon receptor gene IFNAR2. We identified potential targets for repurposing of licensed medications: using Mendelian randomization, we found evidence that low expression of IFNAR2, or high expression of TYK2, are associated with life-threatening disease; and transcriptome-wide association in lung tissue revealed that high expression of the monocyte–macrophage chemotactic receptor CCR2 is associated with severe COVID-19. Our results identify robust genetic signals relating to key host antiviral defence mechanisms and mediators of inflammatory organ damage in COVID-19. Both mechanisms may be amenable to targeted treatment with existing drugs. However, large-scale randomized clinical trials will be essential before any change to clinical practice.</t>
+  </si>
+  <si>
     <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUB25</t>
   </si>
   <si>
     <t>PUB25</t>
   </si>
   <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBLICATIONS_COLLECTION</t>
-  </si>
-  <si>
     <t>Global human-made mass exceeds all living biomass</t>
   </si>
   <si>
-    <t>DataPaper</t>
-  </si>
-  <si>
     <t>https://doi.org/10.1038/s41586-020-3010-5</t>
   </si>
   <si>
@@ -547,9 +554,6 @@
     <t>Global human-made mass exceeds all living biomass for testing purposes</t>
   </si>
   <si>
-    <t>Registered</t>
-  </si>
-  <si>
     <t>2020-12-09 14:43:20 +0000</t>
   </si>
   <si>
@@ -586,39 +590,9 @@
     <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBCREA27</t>
   </si>
   <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBPUB26</t>
-  </si>
-  <si>
     <t>Quantum computational advantage or supremacy is a long-anticipated milestone toward practical quantum computers. Recent work claimed to have reached this point, but subsequent work managed to speed up the classical simulation and pointed toward a sample size–dependent loophole. Quantum computational advantage, rather than being a one-shot experimental proof, will be the result of a long-term competition between quantum devices and classical simulation. Zhong et al. sent 50 indistinguishable single-mode squeezed states into a 100-mode ultralow-loss interferometer and sampled the output using 100 high-efficiency single-photon detectors. By obtaining up to 76-photon coincidence, yielding a state space dimension of about 1030, they measured a sampling rate that is about 1014-fold faster than using state-of-the-art classical simulation strategies and supercomputers.</t>
   </si>
   <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUB29</t>
-  </si>
-  <si>
-    <t>PUB29</t>
-  </si>
-  <si>
-    <t>Genetic mechanisms of critical illness in COVID-19</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.1038/s41586-020-03065-y</t>
-  </si>
-  <si>
-    <t>https://www.nature.com/articles/s41586-020-03065-y#citeas</t>
-  </si>
-  <si>
-    <t>Genetic mechanisms of critical illness in COVID-19 for testing purposes</t>
-  </si>
-  <si>
-    <t>2020-12-11 14:48:55 +0000</t>
-  </si>
-  <si>
-    <t>/PUBLICATIONS/PUBLIC_REPOSITORIES/PUBCREA23</t>
-  </si>
-  <si>
-    <t>Host-mediated lung inflammation is present1, and drives mortality2, in the critical illness caused by coronavirus disease 2019 (COVID-19). Host genetic variants associated with critical illness may identify mechanistic targets for therapeutic development3. Here we report the results of the GenOMICC (Genetics Of Mortality In Critical Care) genome-wide association study in 2,244 critically ill patients with COVID-19 from 208 UK intensive care units. We have identified and replicated the following new genome-wide significant associations: on chromosome 12q24.13 (rs10735079, P = 1.65 × 10−8) in a gene cluster that encodes antiviral restriction enzyme activators (OAS1, OAS2 and OAS3); on chromosome 19p13.2 (rs74956615, P = 2.3 × 10−8) near the gene that encodes tyrosine kinase 2 (TYK2); on chromosome 19p13.3 (rs2109069, P = 3.98 ×  10−12) within the gene that encodes dipeptidyl peptidase 9 (DPP9); and on chromosome 21q22.1 (rs2236757, P = 4.99 × 10−8) in the interferon receptor gene IFNAR2. We identified potential targets for repurposing of licensed medications: using Mendelian randomization, we found evidence that low expression of IFNAR2, or high expression of TYK2, are associated with life-threatening disease; and transcriptome-wide association in lung tissue revealed that high expression of the monocyte–macrophage chemotactic receptor CCR2 is associated with severe COVID-19. Our results identify robust genetic signals relating to key host antiviral defence mechanisms and mediators of inflammatory organ damage in COVID-19. Both mechanisms may be amenable to targeted treatment with existing drugs. However, large-scale randomized clinical trials will be essential before any change to clinical practice.</t>
-  </si>
-  <si>
     <t>PUBCREA27</t>
   </si>
   <si>
@@ -634,6 +608,24 @@
     <t>Han-Sen Zhong</t>
   </si>
   <si>
+    <t>PUBCREA23</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-2423-3090</t>
+  </si>
+  <si>
+    <t>https://orcid.org/</t>
+  </si>
+  <si>
+    <t>Erola Pairo-Castineira</t>
+  </si>
+  <si>
+    <t>Pairo-Castineira</t>
+  </si>
+  <si>
+    <t>Erola</t>
+  </si>
+  <si>
     <t>PUBCREA22</t>
   </si>
   <si>
@@ -646,24 +638,6 @@
     <t>Elhacham</t>
   </si>
   <si>
-    <t>PUBCREA23</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0002-2423-3090</t>
-  </si>
-  <si>
-    <t>https://orcid.org/</t>
-  </si>
-  <si>
-    <t>Erola Pairo-Castineira</t>
-  </si>
-  <si>
-    <t>Pairo-Castineira</t>
-  </si>
-  <si>
-    <t>Erola</t>
-  </si>
-  <si>
     <t>PUBPUB26</t>
   </si>
   <si>
@@ -688,22 +662,22 @@
     <t>Experiment type</t>
   </si>
   <si>
+    <t>PUBLICATIONS_PUBLISHER_COLLECTION</t>
+  </si>
+  <si>
+    <t>Publications Publisher Collection</t>
+  </si>
+  <si>
+    <t>PUBLICATIONS_CREATOR_COLLECTION</t>
+  </si>
+  <si>
+    <t>Publications creator collection</t>
+  </si>
+  <si>
     <t>PUBLICATIONS_COLLECTION</t>
   </si>
   <si>
     <t>Publications Collection</t>
-  </si>
-  <si>
-    <t>PUBLICATIONS_CREATOR_COLLECTION</t>
-  </si>
-  <si>
-    <t>Publications creator collection</t>
-  </si>
-  <si>
-    <t>PUBLICATIONS_PUBLISHER_COLLECTION</t>
-  </si>
-  <si>
-    <t>Publications Publisher Collection</t>
   </si>
 </sst>
 </file>
@@ -1260,18 +1234,18 @@
         <v>9</v>
       </c>
       <c r="Q15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="R15" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="R15" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="S15" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>5</v>
@@ -1286,7 +1260,7 @@
         <v>44</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>46</v>
@@ -1295,7 +1269,7 @@
         <v>11</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>11</v>
@@ -1319,18 +1293,18 @@
         <v>9</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>5</v>
@@ -1345,7 +1319,7 @@
         <v>44</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>46</v>
@@ -1354,7 +1328,7 @@
         <v>11</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>11</v>
@@ -1378,18 +1352,18 @@
         <v>9</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>5</v>
@@ -1404,7 +1378,7 @@
         <v>44</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>46</v>
@@ -1413,7 +1387,7 @@
         <v>11</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>11</v>
@@ -1448,7 +1422,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>5</v>
@@ -1463,7 +1437,7 @@
         <v>44</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>46</v>
@@ -1472,7 +1446,7 @@
         <v>11</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>11</v>
@@ -1507,7 +1481,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>5</v>
@@ -1522,7 +1496,7 @@
         <v>44</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>46</v>
@@ -1531,7 +1505,7 @@
         <v>11</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>11</v>
@@ -1603,7 +1577,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -1618,16 +1592,16 @@
         <v>11</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>11</v>
@@ -1694,7 +1668,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>5</v>
@@ -1709,7 +1683,7 @@
         <v>44</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>46</v>
@@ -1718,7 +1692,7 @@
         <v>11</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>11</v>
@@ -1742,18 +1716,18 @@
         <v>9</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>5</v>
@@ -1801,18 +1775,18 @@
         <v>9</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>5</v>
@@ -1827,7 +1801,7 @@
         <v>44</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>46</v>
@@ -1836,7 +1810,7 @@
         <v>11</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>11</v>
@@ -1860,13 +1834,13 @@
         <v>9</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>86</v>
+        <v>11</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29">
@@ -1967,7 +1941,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>9</v>
@@ -1982,16 +1956,16 @@
         <v>11</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>11</v>
@@ -2109,7 +2083,7 @@
         <v>47</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>91</v>
+        <v>55</v>
       </c>
       <c r="S35" s="1" t="s">
         <v>49</v>
@@ -2117,7 +2091,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>5</v>
@@ -2132,7 +2106,7 @@
         <v>44</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>46</v>
@@ -2141,7 +2115,7 @@
         <v>11</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>11</v>
@@ -2165,18 +2139,18 @@
         <v>9</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>5</v>
@@ -2191,7 +2165,7 @@
         <v>44</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>46</v>
@@ -2200,7 +2174,7 @@
         <v>11</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>11</v>
@@ -2235,7 +2209,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>5</v>
@@ -2250,7 +2224,7 @@
         <v>44</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>46</v>
@@ -2259,7 +2233,7 @@
         <v>11</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>11</v>
@@ -2283,18 +2257,18 @@
         <v>9</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="R38" s="1" t="s">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>5</v>
@@ -2309,16 +2283,16 @@
         <v>44</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>11</v>
@@ -2345,7 +2319,7 @@
         <v>47</v>
       </c>
       <c r="R39" s="1" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="S39" s="1" t="s">
         <v>49</v>
@@ -2353,7 +2327,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>5</v>
@@ -2401,18 +2375,18 @@
         <v>9</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>5</v>
@@ -2427,7 +2401,7 @@
         <v>44</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="G41" s="1" t="s">
         <v>46</v>
@@ -2436,7 +2410,7 @@
         <v>11</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="J41" s="1" t="s">
         <v>11</v>
@@ -2460,18 +2434,18 @@
         <v>9</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="R41" s="1" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>5</v>
@@ -2486,16 +2460,16 @@
         <v>11</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="J42" s="1" t="s">
         <v>11</v>
@@ -2530,7 +2504,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>9</v>
@@ -2545,7 +2519,7 @@
         <v>44</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>46</v>
@@ -2554,7 +2528,7 @@
         <v>11</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>11</v>
@@ -2578,18 +2552,18 @@
         <v>9</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>60</v>
+        <v>106</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>62</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>9</v>
@@ -2604,7 +2578,7 @@
         <v>44</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>46</v>
@@ -2613,7 +2587,7 @@
         <v>11</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="J44" s="1" t="s">
         <v>11</v>
@@ -2637,18 +2611,18 @@
         <v>9</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>9</v>
@@ -2663,16 +2637,16 @@
         <v>44</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="J45" s="1" t="s">
         <v>11</v>
@@ -2696,18 +2670,18 @@
         <v>9</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>47</v>
+        <v>115</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>49</v>
+        <v>117</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>9</v>
@@ -2722,16 +2696,16 @@
         <v>44</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H46" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="J46" s="1" t="s">
         <v>11</v>
@@ -2755,18 +2729,18 @@
         <v>9</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="R46" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="S46" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>9</v>
@@ -2781,16 +2755,16 @@
         <v>44</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="J47" s="1" t="s">
         <v>11</v>
@@ -2814,18 +2788,18 @@
         <v>9</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="R47" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>9</v>
@@ -2840,7 +2814,7 @@
         <v>44</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>46</v>
@@ -2849,7 +2823,7 @@
         <v>11</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="J48" s="1" t="s">
         <v>11</v>
@@ -2873,18 +2847,18 @@
         <v>9</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="R48" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51">
@@ -2912,7 +2886,7 @@
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>9</v>
@@ -3006,7 +2980,7 @@
         <v>5</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>54</v>
@@ -3053,7 +3027,7 @@
     </row>
     <row r="55">
       <c r="A55" s="4" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>5</v>
@@ -3065,10 +3039,10 @@
         <v>5</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G55" s="4" t="s">
         <v>46</v>
@@ -3077,7 +3051,7 @@
         <v>11</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="J55" s="4" t="s">
         <v>11</v>
@@ -3112,7 +3086,7 @@
     </row>
     <row r="56">
       <c r="A56" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>5</v>
@@ -3124,19 +3098,19 @@
         <v>5</v>
       </c>
       <c r="E56" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F56" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="F56" s="4" t="s">
-        <v>144</v>
-      </c>
       <c r="G56" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H56" s="4" t="s">
         <v>4</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="J56" s="4" t="s">
         <v>11</v>
@@ -3171,7 +3145,7 @@
     </row>
     <row r="58">
       <c r="A58" s="14" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="59">
@@ -3184,15 +3158,15 @@
     </row>
     <row r="60">
       <c r="A60" s="13" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="17" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63">
@@ -3206,44 +3180,44 @@
         <v>3</v>
       </c>
       <c r="D63" s="17" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="16" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C64" s="16" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D64" s="16" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="23" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="23" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="22" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="23" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B69" s="23" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C69" s="23" t="s">
         <v>52</v>
@@ -3252,61 +3226,61 @@
         <v>1</v>
       </c>
       <c r="E69" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F69" s="23" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G69" s="23" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H69" s="23" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I69" s="23" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J69" s="23" t="s">
         <v>54</v>
       </c>
       <c r="K69" s="23" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="L69" s="23" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="M69" s="23" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="N69" s="23" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="O69" s="23" t="s">
         <v>3</v>
       </c>
       <c r="P69" s="23" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="Q69" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="R69" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="S69" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="R69" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="S69" s="23" t="s">
-        <v>117</v>
-      </c>
       <c r="T69" s="23" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="U69" s="23" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="V69" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="W69" s="23" t="s">
         <v>128</v>
-      </c>
-      <c r="W69" s="23" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="70">
@@ -3317,67 +3291,67 @@
         <v>9</v>
       </c>
       <c r="C70" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="D70" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E70" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F70" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="G70" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="H70" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="I70" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="J70" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="K70" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="L70" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="M70" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="D70" s="23" t="s">
+      <c r="N70" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="E70" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F70" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="G70" s="23" t="s">
+      <c r="O70" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="H70" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="I70" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="J70" s="23" t="s">
+      <c r="P70" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q70" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="R70" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="K70" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="L70" s="23" t="s">
+      <c r="S70" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="T70" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="M70" s="23" t="s">
+      <c r="U70" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="N70" s="23" t="s">
+      <c r="V70" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="O70" s="23" t="s">
+      <c r="W70" s="23" t="s">
         <v>170</v>
-      </c>
-      <c r="P70" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q70" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="R70" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="S70" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="T70" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="U70" s="23" t="s">
-        <v>173</v>
-      </c>
-      <c r="V70" s="23" t="s">
-        <v>174</v>
-      </c>
-      <c r="W70" s="23" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="71">
@@ -3388,67 +3362,67 @@
         <v>9</v>
       </c>
       <c r="C71" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="D71" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="E71" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F71" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="G71" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="H71" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="I71" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="J71" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="K71" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="L71" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="M71" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="N71" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="O71" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="D71" s="23" t="s">
+      <c r="P71" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q71" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="R71" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="S71" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="T71" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="E71" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F71" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="G71" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="H71" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="I71" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="J71" s="23" t="s">
+      <c r="U71" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="K71" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="L71" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="M71" s="23" t="s">
+      <c r="V71" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="N71" s="23" t="s">
+      <c r="W71" s="23" t="s">
         <v>180</v>
-      </c>
-      <c r="O71" s="23" t="s">
-        <v>181</v>
-      </c>
-      <c r="P71" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q71" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="R71" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="S71" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="T71" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="U71" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="V71" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="W71" s="23" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="72">
@@ -3459,77 +3433,77 @@
         <v>9</v>
       </c>
       <c r="C72" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="D72" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="E72" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F72" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="G72" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="H72" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="I72" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="J72" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="K72" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="L72" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="M72" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="N72" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="O72" s="23" t="s">
         <v>186</v>
       </c>
-      <c r="D72" s="23" t="s">
+      <c r="P72" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q72" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="R72" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="S72" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="T72" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="E72" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F72" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="G72" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="H72" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="I72" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="J72" s="23" t="s">
+      <c r="U72" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="K72" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="L72" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="M72" s="23" t="s">
+      <c r="V72" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="W72" s="23" t="s">
         <v>189</v>
-      </c>
-      <c r="N72" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="O72" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="P72" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q72" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="R72" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="S72" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="T72" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="U72" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="V72" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="W72" s="23" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="23" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="23" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="76">
@@ -3539,10 +3513,10 @@
     </row>
     <row r="77">
       <c r="A77" s="23" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C77" s="23" t="s">
         <v>52</v>
@@ -3551,19 +3525,19 @@
         <v>1</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G77" s="23" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H77" s="23" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J77" s="23" t="s">
         <v>45</v>
@@ -3575,19 +3549,19 @@
         <v>54</v>
       </c>
       <c r="M77" s="23" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N77" s="23" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="O77" s="23" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="P77" s="23" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="Q77" s="23" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="78">
@@ -3598,19 +3572,19 @@
         <v>9</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="G78" s="23" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="H78" s="23" t="s">
         <v>11</v>
@@ -3619,13 +3593,13 @@
         <v>11</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="K78" s="23" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="L78" s="23" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="M78" s="23" t="s">
         <v>11</v>
@@ -3651,40 +3625,40 @@
         <v>9</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D79" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="E79" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F79" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="G79" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="H79" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="I79" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="J79" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="K79" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="L79" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="M79" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="N79" s="23" t="s">
         <v>200</v>
-      </c>
-      <c r="E79" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F79" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="G79" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="H79" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="I79" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="J79" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="K79" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="L79" s="23" t="s">
-        <v>201</v>
-      </c>
-      <c r="M79" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="N79" s="23" t="s">
-        <v>203</v>
       </c>
       <c r="O79" s="23" t="s">
         <v>11</v>
@@ -3704,40 +3678,40 @@
         <v>9</v>
       </c>
       <c r="C80" s="23" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="D80" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="E80" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F80" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="G80" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="H80" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="I80" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="J80" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="K80" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="L80" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="M80" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="N80" s="23" t="s">
         <v>204</v>
-      </c>
-      <c r="E80" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F80" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="G80" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="H80" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="I80" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="J80" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="K80" s="23" t="s">
-        <v>206</v>
-      </c>
-      <c r="L80" s="23" t="s">
-        <v>207</v>
-      </c>
-      <c r="M80" s="23" t="s">
-        <v>208</v>
-      </c>
-      <c r="N80" s="23" t="s">
-        <v>209</v>
       </c>
       <c r="O80" s="23" t="s">
         <v>11</v>
@@ -3751,25 +3725,25 @@
     </row>
     <row r="82">
       <c r="A82" s="23" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="23" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="23" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B85" s="23" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C85" s="23" t="s">
         <v>52</v>
@@ -3778,28 +3752,28 @@
         <v>1</v>
       </c>
       <c r="E85" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F85" s="23" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G85" s="23" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H85" s="23" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I85" s="23" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J85" s="23" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K85" s="23" t="s">
         <v>51</v>
       </c>
       <c r="L85" s="23" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="M85" s="23" t="s">
         <v>54</v>
@@ -3813,19 +3787,19 @@
         <v>9</v>
       </c>
       <c r="C86" s="23" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="D86" s="23" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E86" s="23" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F86" s="23" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="G86" s="23" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="H86" s="23" t="s">
         <v>11</v>
@@ -3834,7 +3808,7 @@
         <v>11</v>
       </c>
       <c r="J86" s="23" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K86" s="23" t="s">
         <v>11</v>
@@ -3843,7 +3817,7 @@
         <v>11</v>
       </c>
       <c r="M86" s="23" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="87">
@@ -3854,19 +3828,19 @@
         <v>9</v>
       </c>
       <c r="C87" s="23" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D87" s="23" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="E87" s="23" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F87" s="23" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="G87" s="23" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="H87" s="23" t="s">
         <v>11</v>
@@ -3875,7 +3849,7 @@
         <v>11</v>
       </c>
       <c r="J87" s="23" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="K87" s="23" t="s">
         <v>11</v>
@@ -3884,22 +3858,22 @@
         <v>11</v>
       </c>
       <c r="M87" s="23" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="20" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="20" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="19" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="92">
@@ -3910,50 +3884,50 @@
         <v>1</v>
       </c>
       <c r="C92" s="20" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D92" s="20" t="s">
         <v>54</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F92" s="20" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="20" t="s">
-        <v>165</v>
+        <v>206</v>
       </c>
       <c r="B93" s="20" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D93" s="20" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E93" s="20" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="F93" s="20" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="20" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B94" s="20" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D94" s="20" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E94" s="20" t="s">
         <v>25</v>
@@ -3964,22 +3938,22 @@
     </row>
     <row r="95">
       <c r="A95" s="20" t="s">
-        <v>211</v>
+        <v>160</v>
       </c>
       <c r="B95" s="20" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C95" s="20" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D95" s="20" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="E95" s="20" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F95" s="20" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>